<commit_message>
docs(QA): integrar 50 objetivos OLC 2025 al cruce temático completo
Los 50 objetivos del OLC Course Review Scorecard 2025 ahora están al
mismo nivel que OSCQR, QM y Sepúlveda en el xlsx:

- Cruce Temático: 219 filas (OSCQR 50 + OLC 2025 50 + QM 42 + Sepúlveda 77)
- OLC 2025 en azul claro, con nivel Esencial/Avanzado/Entrega
- Resumen por Tema: reconstruido con 4 fuentes y consenso X/4
- Leyenda: actualizada con entrada OLC 2025 y color azul

Consenso mejorado: 10 temas ahora tienen 4/4 fuentes (antes 3/3 max)
Temas exclusivos UMCE confirmados: T15 (sincrónica), T14 (privacidad
profunda) siguen sin cobertura OLC 2025

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/espacio-aprendizaje/indicadores-cruce-tematico.xlsx
+++ b/docs/espacio-aprendizaje/indicadores-cruce-tematico.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cruce Tematico'!$A$1:$I$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cruce Tematico'!$A$1:$I$220</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Propuesta Consolidada'!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,7 +44,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
         <bgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEDC8"/>
+        <bgColor rgb="00DCEDC8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -178,6 +184,19 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I170"/>
+  <dimension ref="A1:I220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8546,8 +8565,2358 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Objetivos y resultados de aprendizaje</t>
+        </is>
+      </c>
+      <c r="C171" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D171" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-1</t>
+        </is>
+      </c>
+      <c r="E171" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F171" s="22" t="inlineStr">
+        <is>
+          <t>Los objetivos y/o resultados del aprendizaje son específicos, mensurables y están claramente definidos.</t>
+        </is>
+      </c>
+      <c r="G171" s="22" t="inlineStr">
+        <is>
+          <t>Los objetivos y/o resultados del aprendizaje son específicos, mensurables y están claramente definidos.</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I171" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Requisitos tecnológicos y competencias digitales</t>
+        </is>
+      </c>
+      <c r="C172" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D172" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-2</t>
+        </is>
+      </c>
+      <c r="E172" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F172" s="22" t="inlineStr">
+        <is>
+          <t>El curso enumera todos los materiales de aprendizaje necesarios, incluidas las herramientas tecnológicas.</t>
+        </is>
+      </c>
+      <c r="G172" s="22" t="inlineStr">
+        <is>
+          <t>El curso enumera todos los materiales de aprendizaje necesarios, incluidas las herramientas tecnológicas.</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I172" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C173" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D173" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-3</t>
+        </is>
+      </c>
+      <c r="E173" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F173" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona horas de oficina, preferencias de comunicación y tiempos de respuesta.</t>
+        </is>
+      </c>
+      <c r="G173" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona horas de oficina, preferencias de comunicación y tiempos de respuesta.</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Soporte al estudiante y servicios institucionales</t>
+        </is>
+      </c>
+      <c r="C174" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D174" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-4</t>
+        </is>
+      </c>
+      <c r="E174" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F174" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona recursos de soporte técnico y ayuda para problemas técnicos comunes.</t>
+        </is>
+      </c>
+      <c r="G174" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona recursos de soporte técnico y ayuda para problemas técnicos comunes.</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I174" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Requisitos tecnológicos y competencias digitales</t>
+        </is>
+      </c>
+      <c r="C175" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D175" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-5</t>
+        </is>
+      </c>
+      <c r="E175" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F175" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye guías o tutoriales paso a paso para todas las tecnologías necesarias.</t>
+        </is>
+      </c>
+      <c r="G175" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye guías o tutoriales paso a paso para todas las tecnologías necesarias.</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I175" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Políticas institucionales y normas académicas</t>
+        </is>
+      </c>
+      <c r="C176" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D176" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-6</t>
+        </is>
+      </c>
+      <c r="E176" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F176" s="22" t="inlineStr">
+        <is>
+          <t>El curso define las políticas de calificación, las expectativas de integridad académica y las políticas sobre retrasos.</t>
+        </is>
+      </c>
+      <c r="G176" s="22" t="inlineStr">
+        <is>
+          <t>El curso define las políticas de calificación, las expectativas de integridad académica y las políticas sobre retrasos.</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Accesibilidad multimodal y DUA</t>
+        </is>
+      </c>
+      <c r="C177" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D177" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-7</t>
+        </is>
+      </c>
+      <c r="E177" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F177" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona una declaración de accesibilidad y los pasos para solicitar adaptaciones.</t>
+        </is>
+      </c>
+      <c r="G177" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona una declaración de accesibilidad y los pasos para solicitar adaptaciones.</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I177" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Soporte al estudiante y servicios institucionales</t>
+        </is>
+      </c>
+      <c r="C178" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D178" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-8</t>
+        </is>
+      </c>
+      <c r="E178" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F178" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye información sobre los servicios de apoyo al estudiante y otros servicios.</t>
+        </is>
+      </c>
+      <c r="G178" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye información sobre los servicios de apoyo al estudiante y otros servicios.</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I178" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Bienvenida, orientación e información del curso</t>
+        </is>
+      </c>
+      <c r="C179" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D179" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-9</t>
+        </is>
+      </c>
+      <c r="E179" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F179" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un calendario con las fechas de entrega de todas las tareas y actividades.</t>
+        </is>
+      </c>
+      <c r="G179" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un calendario con las fechas de entrega de todas las tareas y actividades.</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I179" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C180" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D180" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-10</t>
+        </is>
+      </c>
+      <c r="E180" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F180" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un debate introductorio y directrices para la interacción de los estudiantes.</t>
+        </is>
+      </c>
+      <c r="G180" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un debate introductorio y directrices para la interacción de los estudiantes.</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I180" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Navegación, diseño y estructura visual</t>
+        </is>
+      </c>
+      <c r="C181" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D181" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-11</t>
+        </is>
+      </c>
+      <c r="E181" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F181" s="22" t="inlineStr">
+        <is>
+          <t>La navegación y el diseño del sitio del curso son claros y coherentes.</t>
+        </is>
+      </c>
+      <c r="G181" s="22" t="inlineStr">
+        <is>
+          <t>La navegación y el diseño del sitio del curso son claros y coherentes.</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I181" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Contenidos y materiales instruccionales</t>
+        </is>
+      </c>
+      <c r="C182" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D182" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-12</t>
+        </is>
+      </c>
+      <c r="E182" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F182" s="22" t="inlineStr">
+        <is>
+          <t>Los vídeos y otros contenidos multimedia son de calidad y duración adecuadas.</t>
+        </is>
+      </c>
+      <c r="G182" s="22" t="inlineStr">
+        <is>
+          <t>Los vídeos y otros contenidos multimedia son de calidad y duración adecuadas.</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I182" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>Contenidos y materiales instruccionales</t>
+        </is>
+      </c>
+      <c r="C183" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D183" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-13</t>
+        </is>
+      </c>
+      <c r="E183" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F183" s="22" t="inlineStr">
+        <is>
+          <t>El contenido del curso está actualizado, es relevante y está vinculado a objetivos de aprendizaje específicos.</t>
+        </is>
+      </c>
+      <c r="G183" s="22" t="inlineStr">
+        <is>
+          <t>El contenido del curso está actualizado, es relevante y está vinculado a objetivos de aprendizaje específicos.</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I183" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C184" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D184" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-14</t>
+        </is>
+      </c>
+      <c r="E184" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F184" s="22" t="inlineStr">
+        <is>
+          <t>El sitio del curso proporciona un libro de calificaciones organizado que incluye todas las evaluaciones.</t>
+        </is>
+      </c>
+      <c r="G184" s="22" t="inlineStr">
+        <is>
+          <t>El sitio del curso proporciona un libro de calificaciones organizado que incluye todas las evaluaciones.</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I184" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C185" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D185" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-15</t>
+        </is>
+      </c>
+      <c r="E185" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F185" s="22" t="inlineStr">
+        <is>
+          <t>El curso incorpora evaluaciones formativas de baja exigencia para un compromiso frecuente.</t>
+        </is>
+      </c>
+      <c r="G185" s="22" t="inlineStr">
+        <is>
+          <t>El curso incorpora evaluaciones formativas de baja exigencia para un compromiso frecuente.</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I185" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C186" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D186" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-16</t>
+        </is>
+      </c>
+      <c r="E186" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F186" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona un enfoque de andamiaje para las evaluaciones sumativas.</t>
+        </is>
+      </c>
+      <c r="G186" s="22" t="inlineStr">
+        <is>
+          <t>El curso proporciona un enfoque de andamiaje para las evaluaciones sumativas.</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I186" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>Contenidos y materiales instruccionales</t>
+        </is>
+      </c>
+      <c r="C187" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D187" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-17</t>
+        </is>
+      </c>
+      <c r="E187" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F187" s="22" t="inlineStr">
+        <is>
+          <t>Todos los módulos, tareas y actividades incluyen instrucciones claras y detalladas.</t>
+        </is>
+      </c>
+      <c r="G187" s="22" t="inlineStr">
+        <is>
+          <t>Todos los módulos, tareas y actividades incluyen instrucciones claras y detalladas.</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I187" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C188" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D188" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-18</t>
+        </is>
+      </c>
+      <c r="E188" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F188" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye rúbricas para todas las tareas y evaluaciones.</t>
+        </is>
+      </c>
+      <c r="G188" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye rúbricas para todas las tareas y evaluaciones.</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I188" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>Bienestar, cuidados digitales y corresponsabilidad</t>
+        </is>
+      </c>
+      <c r="C189" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D189" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-19</t>
+        </is>
+      </c>
+      <c r="E189" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F189" s="22" t="inlineStr">
+        <is>
+          <t>La carga de trabajo del curso es equilibrada y apropiada para la disciplina y el nivel del curso.</t>
+        </is>
+      </c>
+      <c r="G189" s="22" t="inlineStr">
+        <is>
+          <t>La carga de trabajo del curso es equilibrada y apropiada para la disciplina y el nivel del curso.</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I189" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Funcionalidad técnica de la plataforma</t>
+        </is>
+      </c>
+      <c r="C190" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D190" s="22" t="inlineStr">
+        <is>
+          <t>OLC-E-20</t>
+        </is>
+      </c>
+      <c r="E190" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Esencial</t>
+        </is>
+      </c>
+      <c r="F190" s="22" t="inlineStr">
+        <is>
+          <t>Los materiales del curso no contienen enlaces rotos, errores ortográficos ni información incorrecta.</t>
+        </is>
+      </c>
+      <c r="G190" s="22" t="inlineStr">
+        <is>
+          <t>Los materiales del curso no contienen enlaces rotos, errores ortográficos ni información incorrecta.</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Esencial</t>
+        </is>
+      </c>
+      <c r="I190" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Objetivos y resultados de aprendizaje</t>
+        </is>
+      </c>
+      <c r="C191" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D191" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-1</t>
+        </is>
+      </c>
+      <c r="E191" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F191" s="22" t="inlineStr">
+        <is>
+          <t>Los objetivos y/o resultados de aprendizaje del curso utilizan un lenguaje centrado en el alumno.</t>
+        </is>
+      </c>
+      <c r="G191" s="22" t="inlineStr">
+        <is>
+          <t>Los objetivos y/o resultados de aprendizaje del curso utilizan un lenguaje centrado en el alumno.</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I191" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Requisitos tecnológicos y competencias digitales</t>
+        </is>
+      </c>
+      <c r="C192" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D192" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-2</t>
+        </is>
+      </c>
+      <c r="E192" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F192" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye una lista de comprobación tecnológica previa al curso y un cuestionario de preparación en línea.</t>
+        </is>
+      </c>
+      <c r="G192" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye una lista de comprobación tecnológica previa al curso y un cuestionario de preparación en línea.</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I192" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Bienvenida, orientación e información del curso</t>
+        </is>
+      </c>
+      <c r="C193" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D193" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-3</t>
+        </is>
+      </c>
+      <c r="E193" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F193" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un módulo de orientación, un vídeo o una guía para navegar por el curso.</t>
+        </is>
+      </c>
+      <c r="G193" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un módulo de orientación, un vídeo o una guía para navegar por el curso.</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I193" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Políticas institucionales y normas académicas</t>
+        </is>
+      </c>
+      <c r="C194" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D194" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-4</t>
+        </is>
+      </c>
+      <c r="E194" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F194" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye directrices explícitas para el uso de la IA generativa.</t>
+        </is>
+      </c>
+      <c r="G194" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye directrices explícitas para el uso de la IA generativa.</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I194" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>Recursos educativos abiertos (REA) y licencias</t>
+        </is>
+      </c>
+      <c r="C195" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D195" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-5</t>
+        </is>
+      </c>
+      <c r="E195" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F195" s="22" t="inlineStr">
+        <is>
+          <t>El curso utiliza exclusivamente materiales de bajo coste o gratuitos.</t>
+        </is>
+      </c>
+      <c r="G195" s="22" t="inlineStr">
+        <is>
+          <t>El curso utiliza exclusivamente materiales de bajo coste o gratuitos.</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I195" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C196" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D196" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-6</t>
+        </is>
+      </c>
+      <c r="E196" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F196" s="22" t="inlineStr">
+        <is>
+          <t>El curso ofrece múltiples vías para que los alumnos alcancen los objetivos de aprendizaje.</t>
+        </is>
+      </c>
+      <c r="G196" s="22" t="inlineStr">
+        <is>
+          <t>El curso ofrece múltiples vías para que los alumnos alcancen los objetivos de aprendizaje.</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I196" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>Perspectiva de género, equidad y trato no discriminatorio</t>
+        </is>
+      </c>
+      <c r="C197" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D197" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-7</t>
+        </is>
+      </c>
+      <c r="E197" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F197" s="22" t="inlineStr">
+        <is>
+          <t>El contenido incluye ejemplos que representan a una amplia gama de alumnos.</t>
+        </is>
+      </c>
+      <c r="G197" s="22" t="inlineStr">
+        <is>
+          <t>El contenido incluye ejemplos que representan a una amplia gama de alumnos.</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I197" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C198" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D198" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-8</t>
+        </is>
+      </c>
+      <c r="E198" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F198" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un foro en línea para los puntos más confusos o las preguntas sobre el curso.</t>
+        </is>
+      </c>
+      <c r="G198" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye un foro en línea para los puntos más confusos o las preguntas sobre el curso.</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I198" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C199" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D199" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-9</t>
+        </is>
+      </c>
+      <c r="E199" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F199" s="22" t="inlineStr">
+        <is>
+          <t>El curso incorpora estrategias de aprendizaje adaptativo para personalizar el aprendizaje.</t>
+        </is>
+      </c>
+      <c r="G199" s="22" t="inlineStr">
+        <is>
+          <t>El curso incorpora estrategias de aprendizaje adaptativo para personalizar el aprendizaje.</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I199" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Accesibilidad multimodal y DUA</t>
+        </is>
+      </c>
+      <c r="C200" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D200" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-10</t>
+        </is>
+      </c>
+      <c r="E200" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F200" s="22" t="inlineStr">
+        <is>
+          <t>Los materiales de texto cumplen las normas de accesibilidad y diseño universal.</t>
+        </is>
+      </c>
+      <c r="G200" s="22" t="inlineStr">
+        <is>
+          <t>Los materiales de texto cumplen las normas de accesibilidad y diseño universal.</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I200" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Accesibilidad multimodal y DUA</t>
+        </is>
+      </c>
+      <c r="C201" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D201" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-11</t>
+        </is>
+      </c>
+      <c r="E201" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F201" s="22" t="inlineStr">
+        <is>
+          <t>Los vídeos y otros contenidos multimedia cumplen las normas de accesibilidad.</t>
+        </is>
+      </c>
+      <c r="G201" s="22" t="inlineStr">
+        <is>
+          <t>Los vídeos y otros contenidos multimedia cumplen las normas de accesibilidad.</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I201" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C202" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D202" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-12</t>
+        </is>
+      </c>
+      <c r="E202" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F202" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye formas para que los alumnos contribuyan de manera significativa al contenido del curso.</t>
+        </is>
+      </c>
+      <c r="G202" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye formas para que los alumnos contribuyan de manera significativa al contenido del curso.</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I202" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C203" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D203" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-13</t>
+        </is>
+      </c>
+      <c r="E203" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F203" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye modelos de entregables para las evaluaciones sumativas.</t>
+        </is>
+      </c>
+      <c r="G203" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye modelos de entregables para las evaluaciones sumativas.</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I203" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C204" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D204" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-14</t>
+        </is>
+      </c>
+      <c r="E204" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F204" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye evaluaciones con aplicaciones prácticas de palabras reales.</t>
+        </is>
+      </c>
+      <c r="G204" s="22" t="inlineStr">
+        <is>
+          <t>El curso incluye evaluaciones con aplicaciones prácticas de palabras reales.</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I204" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C205" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D205" s="22" t="inlineStr">
+        <is>
+          <t>OLC-A-15</t>
+        </is>
+      </c>
+      <c r="E205" s="22" t="inlineStr">
+        <is>
+          <t>Diseño Avanzado</t>
+        </is>
+      </c>
+      <c r="F205" s="22" t="inlineStr">
+        <is>
+          <t>El curso apoya la metacognición del alumno mediante actividades periódicas de autorreflexión.</t>
+        </is>
+      </c>
+      <c r="G205" s="22" t="inlineStr">
+        <is>
+          <t>El curso apoya la metacognición del alumno mediante actividades periódicas de autorreflexión.</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Avanzado</t>
+        </is>
+      </c>
+      <c r="I205" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C206" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D206" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-1</t>
+        </is>
+      </c>
+      <c r="E206" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F206" s="22" t="inlineStr">
+        <is>
+          <t>El instructor ofrece una introducción personal al curso.</t>
+        </is>
+      </c>
+      <c r="G206" s="22" t="inlineStr">
+        <is>
+          <t>El instructor ofrece una introducción personal al curso.</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I206" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Competencias docentes para la virtualidad</t>
+        </is>
+      </c>
+      <c r="C207" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D207" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-2</t>
+        </is>
+      </c>
+      <c r="E207" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F207" s="22" t="inlineStr">
+        <is>
+          <t>El instructor publica módulos y contenidos en el sitio del curso de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="G207" s="22" t="inlineStr">
+        <is>
+          <t>El instructor publica módulos y contenidos en el sitio del curso de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I207" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C208" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D208" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-3</t>
+        </is>
+      </c>
+      <c r="E208" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F208" s="22" t="inlineStr">
+        <is>
+          <t>El instructor publica anuncios regulares y relevantes en el sitio del curso.</t>
+        </is>
+      </c>
+      <c r="G208" s="22" t="inlineStr">
+        <is>
+          <t>El instructor publica anuncios regulares y relevantes en el sitio del curso.</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I208" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C209" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D209" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-4</t>
+        </is>
+      </c>
+      <c r="E209" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F209" s="22" t="inlineStr">
+        <is>
+          <t>El instructor contribuye significativamente a las actividades y discusiones en línea.</t>
+        </is>
+      </c>
+      <c r="G209" s="22" t="inlineStr">
+        <is>
+          <t>El instructor contribuye significativamente a las actividades y discusiones en línea.</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I209" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C210" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D210" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-5</t>
+        </is>
+      </c>
+      <c r="E210" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F210" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona retroalimentación específica y dirigida sobre las tareas.</t>
+        </is>
+      </c>
+      <c r="G210" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona retroalimentación específica y dirigida sobre las tareas.</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I210" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C211" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D211" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-6</t>
+        </is>
+      </c>
+      <c r="E211" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F211" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona retroalimentación y califica las evaluaciones de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="G211" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona retroalimentación y califica las evaluaciones de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I211" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Competencias docentes para la virtualidad</t>
+        </is>
+      </c>
+      <c r="C212" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D212" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-7</t>
+        </is>
+      </c>
+      <c r="E212" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F212" s="22" t="inlineStr">
+        <is>
+          <t>El profesor se compromete activamente con los alumnos que muestran dificultades en el curso.</t>
+        </is>
+      </c>
+      <c r="G212" s="22" t="inlineStr">
+        <is>
+          <t>El profesor se compromete activamente con los alumnos que muestran dificultades en el curso.</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I212" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C213" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D213" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-8</t>
+        </is>
+      </c>
+      <c r="E213" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F213" s="22" t="inlineStr">
+        <is>
+          <t>El instructor utiliza un lenguaje de apoyo en todos los comentarios y comunicaciones.</t>
+        </is>
+      </c>
+      <c r="G213" s="22" t="inlineStr">
+        <is>
+          <t>El instructor utiliza un lenguaje de apoyo en todos los comentarios y comunicaciones.</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I213" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C214" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D214" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-9</t>
+        </is>
+      </c>
+      <c r="E214" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F214" s="22" t="inlineStr">
+        <is>
+          <t>El instructor anima o incentiva a los alumnos a participar en las horas de oficina.</t>
+        </is>
+      </c>
+      <c r="G214" s="22" t="inlineStr">
+        <is>
+          <t>El instructor anima o incentiva a los alumnos a participar en las horas de oficina.</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I214" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C215" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D215" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-10</t>
+        </is>
+      </c>
+      <c r="E215" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F215" s="22" t="inlineStr">
+        <is>
+          <t>El instructor responde a las comunicaciones y consultas de los estudiantes de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="G215" s="22" t="inlineStr">
+        <is>
+          <t>El instructor responde a las comunicaciones y consultas de los estudiantes de manera oportuna.</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I215" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Competencias docentes para la virtualidad</t>
+        </is>
+      </c>
+      <c r="C216" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D216" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-11</t>
+        </is>
+      </c>
+      <c r="E216" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F216" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona resúmenes al final del módulo basados en las contribuciones de los alumnos.</t>
+        </is>
+      </c>
+      <c r="G216" s="22" t="inlineStr">
+        <is>
+          <t>El instructor proporciona resúmenes al final del módulo basados en las contribuciones de los alumnos.</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I216" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Actividades de aprendizaje e interacción</t>
+        </is>
+      </c>
+      <c r="C217" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D217" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-12</t>
+        </is>
+      </c>
+      <c r="E217" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F217" s="22" t="inlineStr">
+        <is>
+          <t>El instructor fomenta la participación de alumno a alumno en las actividades en línea.</t>
+        </is>
+      </c>
+      <c r="G217" s="22" t="inlineStr">
+        <is>
+          <t>El instructor fomenta la participación de alumno a alumno en las actividades en línea.</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I217" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Competencias docentes para la virtualidad</t>
+        </is>
+      </c>
+      <c r="C218" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D218" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-13</t>
+        </is>
+      </c>
+      <c r="E218" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F218" s="22" t="inlineStr">
+        <is>
+          <t>El instructor ajusta el contenido, las tareas y las fechas en respuesta a las necesidades del alumno.</t>
+        </is>
+      </c>
+      <c r="G218" s="22" t="inlineStr">
+        <is>
+          <t>El instructor ajusta el contenido, las tareas y las fechas en respuesta a las necesidades del alumno.</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I218" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Evaluación, retroalimentación y calificaciones</t>
+        </is>
+      </c>
+      <c r="C219" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D219" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-14</t>
+        </is>
+      </c>
+      <c r="E219" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F219" s="22" t="inlineStr">
+        <is>
+          <t>El instructor solicita la opinión de los alumnos sobre el curso en varios momentos del curso.</t>
+        </is>
+      </c>
+      <c r="G219" s="22" t="inlineStr">
+        <is>
+          <t>El instructor solicita la opinión de los alumnos sobre el curso en varios momentos del curso.</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I219" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Presencia docente e interacción instructor-estudiante</t>
+        </is>
+      </c>
+      <c r="C220" s="22" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="D220" s="22" t="inlineStr">
+        <is>
+          <t>OLC-D-15</t>
+        </is>
+      </c>
+      <c r="E220" s="22" t="inlineStr">
+        <is>
+          <t>Entrega del Curso</t>
+        </is>
+      </c>
+      <c r="F220" s="22" t="inlineStr">
+        <is>
+          <t>El instructor incorpora ejemplos personales para complementar el contenido del curso.</t>
+        </is>
+      </c>
+      <c r="G220" s="22" t="inlineStr">
+        <is>
+          <t>El instructor incorpora ejemplos personales para complementar el contenido del curso.</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>Nivel: Entrega</t>
+        </is>
+      </c>
+      <c r="I220" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I170"/>
+  <autoFilter ref="A1:I220"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11246,18 +13615,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11268,7 +13638,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Grupo tematico</t>
+          <t>Grupo temático</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -11278,32 +13648,37 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>QM</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sepúlveda</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Consenso</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Auto predominante</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Observacion</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Observación</t>
         </is>
       </c>
     </row>
@@ -11322,27 +13697,30 @@
         <v>6</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+        <v>3</v>
+      </c>
+      <c r="G2" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. Las 3 fuentes cubren bienvenida y orientación.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). Bienvenida y orientación cubiertas por todas las fuentes.</t>
         </is>
       </c>
     </row>
@@ -11361,27 +13739,30 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G3" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. QM tiene la cobertura más exhaustiva (5 estándares esenciales).</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). QM y OLC 2025 tienen cobertura más exhaustiva.</t>
         </is>
       </c>
     </row>
@@ -11400,27 +13781,30 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G4" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Consenso parcial. Sepúlveda agrega protocolos IA (D6.1.2), ausentes en marcos internacionales.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). OLC 2025 agrega directrices IA generativa. Sepúlveda agrega protocolos IA educativa (D6.1.2).</t>
         </is>
       </c>
     </row>
@@ -11439,27 +13823,30 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>2/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G5" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>3/4 fuentes</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Consenso. OSCQR y QM cubren requisitos técnicos; Sepúlveda no aborda explícitamente.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 3/4. Sepúlveda no aborda explícitamente. OLC 2025 agrega diagnóstico de preparación previa.</t>
         </is>
       </c>
     </row>
@@ -11478,27 +13865,30 @@
         <v>14</v>
       </c>
       <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G6" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. OSCQR tiene la cobertura más detallada (13 estándares de diseño).</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (3/4). OSCQR tiene la cobertura más detallada (13 estándares). OLC 2025 aporta 1 objetivo.</t>
         </is>
       </c>
     </row>
@@ -11517,27 +13907,30 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>5</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>1/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>2/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Solo Sepúlveda. Funcionalidad técnica (botones, enlaces, pop-ups) es específica de plataforma LMS.</t>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 2/4. Sepúlveda + OLC 2025 (enlaces rotos). Funcionalidad técnica específica de plataforma LMS.</t>
         </is>
       </c>
     </row>
@@ -11556,27 +13949,30 @@
         <v>1</v>
       </c>
       <c r="D8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G8" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. Materiales instruccionales cubiertos por las 3 fuentes.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). Materiales instruccionales cubiertos por todas las fuentes.</t>
         </is>
       </c>
     </row>
@@ -11598,24 +13994,27 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G9" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. REA y copyright cubiertos por las 3 fuentes. Sepúlveda agrega Creative Commons y código abierto.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 3/4. REA y copyright en OSCQR, QM y Sepúlveda. OLC 2025 agrega materiales gratuitos.</t>
         </is>
       </c>
     </row>
@@ -11634,27 +14033,30 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="F10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Alto consenso. Actividades de aprendizaje activo e interacción en las 3 fuentes.</t>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). OLC 2025 agrega aprendizaje adaptativo y co-creación de contenido.</t>
         </is>
       </c>
     </row>
@@ -11673,27 +14075,30 @@
         <v>7</v>
       </c>
       <c r="D11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G11" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. Evaluación es área central en las 3 fuentes. Sepúlveda agrega retroalimentación personalizada.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). OLC 2025 tiene cobertura más amplia: andamiaje, formativas, metacognición, retroalimentación oportuna.</t>
         </is>
       </c>
     </row>
@@ -11712,27 +14117,30 @@
         <v>3</v>
       </c>
       <c r="D12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="F12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Alto consenso. RSI (OSCQR) + plan docente (QM) + tutorías (Sepúlveda).</t>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). OLC 2025 aporta 7 objetivos de entrega docente (la mayor contribución nueva).</t>
         </is>
       </c>
     </row>
@@ -11751,27 +14159,30 @@
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="F13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G13" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. Soporte y servicios institucionales en las 3 fuentes.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). Soporte y servicios institucionales en todas las fuentes.</t>
         </is>
       </c>
     </row>
@@ -11790,27 +14201,30 @@
         <v>4</v>
       </c>
       <c r="D14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="F14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G14" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>4/4 fuentes</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Alto consenso. Accesibilidad cubierta ampliamente. Sepúlveda agrega lengua de signos y Braille.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Alto consenso (4/4). OLC 2025 distingue accesibilidad de texto vs multimedia.</t>
         </is>
       </c>
     </row>
@@ -11829,27 +14243,30 @@
         <v>1</v>
       </c>
       <c r="D15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="F15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="H15" s="25" t="inlineStr">
+        <is>
+          <t>3/4 fuentes</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Consenso parcial. OSCQR y QM mencionan privacidad; Sepúlveda la desarrolla en 4 indicadores.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 2/4. OSCQR y Sepúlveda. QM y OLC 2025 no desarrollan privacidad en profundidad.</t>
         </is>
       </c>
     </row>
@@ -11871,24 +14288,27 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>1/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="G16" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>1/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Solo Sepúlveda. OSCQR y QM no contemplan sesiones sincrónicas.</t>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Solo Sepúlveda. OSCQR, QM y OLC 2025 no contemplan sesiones sincrónicas.</t>
         </is>
       </c>
     </row>
@@ -11907,27 +14327,30 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>7</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>1/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="G17" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>2/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Solo Sepúlveda. Competencias docentes virtuales no están en marcos internacionales como dimensión propia.</t>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 2/4. Sepúlveda + OLC 2025 (entrega del curso). Competencias docentes virtuales.</t>
         </is>
       </c>
     </row>
@@ -11946,27 +14369,30 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>5</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>1/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="G18" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>2/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Solo Sepúlveda. Género y equidad es aporte original UMCE. Gap total en marcos internacionales.</t>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 2/4. Sepúlveda + OLC 2025 (representación diversa). Gap en OSCQR y QM.</t>
         </is>
       </c>
     </row>
@@ -11985,27 +14411,30 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>12</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>1/3 fuentes</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="G19" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>2/4 fuentes</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Solo Sepúlveda. Bienestar digital y corresponsabilidad es aporte original UMCE.</t>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Consenso 2/4. Sepúlveda (principal) + OLC 2025 (carga de trabajo). Bienestar y corresponsabilidad es aporte UMCE.</t>
         </is>
       </c>
     </row>
@@ -12020,7 +14449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12034,6 +14463,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -12077,173 +14507,202 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>OLC 2025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OLC Course Review Scorecard (2025). Libre. 50 objetivos (20 esencial + 15 avanzado + 15 entrega). En español.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Automatizabilidad</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Automatizable: verificable vía Moodle API o scraping (ej: enlace existe, grabación disponible, syllabus presente).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Semi-automatizable: se puede detectar presencia pero no calidad (ej: rúbrica existe, pero no si es buena).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Requiere evaluación humana: juicio cualitativo necesario (ej: lenguaje inclusivo, retroalimentación constructiva).</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Consenso</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>3/3 fuentes</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Las tres fuentes cubren este tema. Fuerte respaldo internacional.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2/3 fuentes</t>
+          <t>3/3 fuentes</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dos fuentes cubren el tema. Respaldo parcial.</t>
+          <t>Las tres fuentes cubren este tema. Fuerte respaldo internacional.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>2/3 fuentes</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dos fuentes cubren el tema. Respaldo parcial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>1/3 fuentes</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Solo una fuente. Puede ser aporte original UMCE (D5, D6, D3.4) o especificidad de plataforma.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Colores filas</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Naranja claro</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Indicador OSCQR</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Violeta claro</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Indicador Quality Matters</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Verde claro</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Indicador Sepúlveda UMCE</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Azul claro</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Indicador OLC 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Propuesta Consolidada</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>QA-XX</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Código del indicador propuesto para el set UMCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Fuentes</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Códigos de los indicadores originales que sustentan el propuesto (ej: OSCQR-1 + QM-1.1 + D3.3.1)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>QA-XX</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Código del indicador propuesto para el set UMCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Códigos de los indicadores originales que sustentan el propuesto (ej: OSCQR-1 + QM-1.1 + D3.3.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>64 indicadores</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Consolidación de 169 originales. Mesa 1 valida pertinencia y claridad de cada uno.</t>
         </is>

</xml_diff>

<commit_message>
fix: renombrar fuente "Sepúlveda UMCE" → "UDFV-UMCE" + corregir proyecto UMC20992 → UMC21992
El marco evaluativo es de la UDFV, no de la investigadora personalmente.
Sepúlveda Parrini se cita como autora en las referencias bibliográficas,
pero la fuente institucional es la Unidad de Desarrollo y Formación Virtual.

- "Sepúlveda UMCE" → "UDFV-UMCE" en xlsx (79 celdas), contexto, insumo
- "UMC20992" → "UMC21992" en todos los archivos:
  contexto, insumo, JSON, xlsx, qa.html, rubrica.html, fundamentos.html
- Título sección 4 del contexto: "Marco Evaluativo UDFV" (no "Sepúlveda")

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/espacio-aprendizaje/indicadores-cruce-tematico.xlsx
+++ b/docs/espacio-aprendizaje/indicadores-cruce-tematico.xlsx
@@ -1086,7 +1086,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -6068,7 +6068,7 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -6162,7 +6162,7 @@
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
@@ -7337,7 +7337,7 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
@@ -7713,7 +7713,7 @@
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
@@ -7948,7 +7948,7 @@
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
@@ -8089,7 +8089,7 @@
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
@@ -8418,7 +8418,7 @@
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
@@ -8512,7 +8512,7 @@
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
@@ -15733,6 +15733,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -15767,12 +15768,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sepúlveda UMCE</t>
+          <t>UDFV-UMCE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Marco Evaluativo Cursos Virtuales UMCE (2024). UMC20992. 77 indicadores.</t>
+          <t>Marco Evaluativo Cursos Virtuales UMCE (2024). UMC21992. 77 indicadores.</t>
         </is>
       </c>
     </row>
@@ -15788,6 +15789,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
@@ -15831,6 +15833,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
@@ -15874,6 +15877,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
@@ -15913,7 +15917,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Indicador Sepúlveda UMCE</t>
+          <t>Indicador UDFV-UMCE</t>
         </is>
       </c>
     </row>
@@ -15929,6 +15933,8 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
@@ -15972,17 +15978,14 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-    </row>
+    <row r="30"/>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
           <t>CNA Chile (5ta fuente)</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="33" t="inlineStr">

</xml_diff>